<commit_message>
Phase 2: import the Fault Log and opening stock; show errors in red
- import_workbook (same signature) now takes faults and stock: FLT numbers
  kept, the supplier in Action Taken becomes a vendor ("lanka pc" ->
  "Lanka PC"), the reporter is matched to the register by name, the FLT
  sequence moves past them. Each consumable's received and issued totals
  become an opening balance, written once.
- The parser reads the Fault Log and Consumables tabs, with warnings for
  rows it skips; the Import page shows the new counts.
- Labels for fault status and cause, service job type, stock movement type.
- The destructive Alert kept its text grey; errors now show red.
- Tests: import.sql, parser and fixture tests.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MqaKRbo6T91YVta8TRbiTW
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample-workbook.xlsx
+++ b/tests/fixtures/sample-workbook.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="93">
   <si>
     <t>Category</t>
   </si>
@@ -296,9 +296,6 @@
   </si>
   <si>
     <t>MOU-0001</t>
-  </si>
-  <si>
-    <t>REORDER</t>
   </si>
 </sst>
 </file>
@@ -1233,13 +1230,15 @@
         <v>22</v>
       </c>
       <c r="E2">
+        <f>C2-D2</f>
         <v>8</v>
       </c>
       <c r="F2">
         <v>10</v>
       </c>
-      <c r="G2" t="s">
-        <v>93</v>
+      <c r="G2" t="str">
+        <f>IF(C2-D2&lt;=F2,"REORDER","OK")</f>
+        <v>REORDER</v>
       </c>
       <c r="H2" t="s">
         <v>40</v>

</xml_diff>